<commit_message>
Versjon 2.5.6 · pensumsjekk av 30 kapitler, MA08 360 dager, rettede PDF-er og app-innhold
</commit_message>
<xml_diff>
--- a/pensum/ma08/MA08_Distribusjon_Regneark_Grossist_eller_direkte.xlsx
+++ b/pensum/ma08/MA08_Distribusjon_Regneark_Grossist_eller_direkte.xlsx
@@ -654,7 +654,7 @@
     <t xml:space="preserve">Lagerandel ved direkte innkjøp</t>
   </si>
   <si>
-    <t xml:space="preserve">Kredittandel som faller bort (kredittdager delt på 365)</t>
+    <t xml:space="preserve">Kredittandel som faller bort (kredittdager delt på 360)</t>
   </si>
   <si>
     <t xml:space="preserve">= Kapital bundet per krone materiell</t>
@@ -1001,12 +1001,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1014,11 +1018,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1026,7 +1030,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1034,15 +1038,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1050,11 +1054,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1066,31 +1070,31 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1098,67 +1102,67 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1426,271 +1430,271 @@
   <dimension ref="A1:C33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>7990000</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>2100000</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>469760</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>7300</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">B5*B6</f>
         <v>799000</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="10" t="n">
-        <f aca="false">B5*B8/365</f>
-        <v>656712.328767123</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="B16" s="11" t="n">
+        <f aca="false">B5*B8/360</f>
+        <v>665833.333333333</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">(B7+B16)*B9</f>
-        <v>275671.232876712</v>
-      </c>
-      <c r="C17" s="7" t="s">
+        <v>276583.333333333</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">B11*B12</f>
         <v>306600</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">B17+B10+B18</f>
-        <v>1052031.23287671</v>
-      </c>
-      <c r="C19" s="7" t="s">
+        <v>1052943.33333333</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <f aca="false">B15-B19</f>
-        <v>-253031.232876712</v>
-      </c>
-      <c r="C21" s="7" t="s">
+        <v>-253943.333333334</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="14" t="n">
         <f aca="false">B19/B5</f>
-        <v>0.131668489721741</v>
-      </c>
-      <c r="C22" s="7" t="s">
+        <v>0.131782644972883</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="str">
+      <c r="A25" s="15" t="str">
         <f aca="false">"Rabatten gir "&amp;TEXT(ROUND(B15,0),"#,##0")&amp;" kroner, men oppgavene dere arver koster "&amp;TEXT(ROUND(B19,0),"#,##0")&amp;" kroner. Netto blir "&amp;TEXT(ROUND(B21,0),"#,##0")&amp;" kroner."</f>
-        <v>Rabatten gir 799,000 kroner, men oppgavene dere arver koster 1,052,031 kroner. Netto blir -253,031 kroner.</v>
-      </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
+        <v>Rabatten gir 799,000 kroner, men oppgavene dere arver koster 1,052,943 kroner. Netto blir -253,943 kroner.</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="str">
+      <c r="A26" s="15" t="str">
         <f aca="false">"Rabatten måtte vært "&amp;TEXT(B22,"0.0 %")&amp;" for at direktekjøpet skulle gå i null."</f>
         <v>Rabatten måtte vært 13.2 % for at direktekjøpet skulle gå i null.</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1720,277 +1724,277 @@
   <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="62"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="21" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="21" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="21" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="21" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="24" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="21" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="21" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="21" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C32" s="21" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="21" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="21" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="19" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="19" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2013,294 +2017,294 @@
   <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="25" t="n">
         <v>9800</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="26" t="n">
         <v>0.1</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="21" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="25" t="n">
+      <c r="B7" s="26" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="26" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="27" t="n">
         <f aca="false">B5*(1-B6)</f>
         <v>8820</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="28" t="n">
         <f aca="false">B12/$B$15</f>
         <v>0.6</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="21" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="27" t="n">
         <f aca="false">B5</f>
         <v>9800</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="29" t="n">
         <f aca="false">B13-B12</f>
         <v>980</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="28" t="n">
         <f aca="false">B13/$B$15</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="21" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="26" t="n">
+      <c r="B14" s="27" t="n">
         <f aca="false">B13*(1+B7)</f>
         <v>11760</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="29" t="n">
         <f aca="false">B14-B13</f>
         <v>1960</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="28" t="n">
         <f aca="false">B14/$B$15</f>
         <v>0.8</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="21" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="28" t="n">
+      <c r="B15" s="29" t="n">
         <f aca="false">B14*(1+B8)</f>
         <v>14700</v>
       </c>
-      <c r="C15" s="26" t="n">
+      <c r="C15" s="27" t="n">
         <f aca="false">B15-B14</f>
         <v>2940</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="28" t="n">
         <f aca="false">B15/$B$15</f>
         <v>1</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="21" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="27" t="n">
+      <c r="B18" s="28" t="n">
         <f aca="false">C13/B13</f>
         <v>0.1</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="21" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B19" s="27" t="n">
+      <c r="B19" s="28" t="n">
         <f aca="false">C14/B13</f>
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="B20" s="27" t="n">
+      <c r="B20" s="28" t="n">
         <f aca="false">C14/B14</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="21" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B23" s="29" t="n">
+      <c r="B23" s="30" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B24" s="29" t="n">
+      <c r="B24" s="30" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="B25" s="30" t="n">
+      <c r="B25" s="31" t="n">
         <f aca="false">B23*B24</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B26" s="30" t="n">
+      <c r="B26" s="31" t="n">
         <f aca="false">B23+B24</f>
         <v>65</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="30" t="n">
+      <c r="B27" s="31" t="n">
         <f aca="false">B25-B26</f>
         <v>935</v>
       </c>
-      <c r="C27" s="27" t="n">
+      <c r="C27" s="28" t="n">
         <f aca="false">B27/B25</f>
         <v>0.935</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="E27" s="21" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="C30" s="31" t="str">
+      <c r="C30" s="32" t="str">
         <f aca="false">IF(AND(B12&lt;B13,B13&lt;B14,B14&lt;B15),"OK — prisen stiger leddvis fra produsent til sluttkunde","AVVIK: et ledd tar negativ margin. Kontroller prosentene i B6 og B7")</f>
         <v>OK — prisen stiger leddvis fra produsent til sluttkunde</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="C31" s="31" t="str">
+      <c r="C31" s="32" t="str">
         <f aca="false">IF(B20&lt;B19,"OK — bruttofortjenesten i prosent av pris er lavere enn avansen i prosent av inntakskost, som den skal","AVVIK: kontroller nevnerne i B19 og B20")</f>
         <v>OK — bruttofortjenesten i prosent av pris er lavere enn avansen i prosent av inntakskost, som den skal</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C32" s="31" t="str">
+      <c r="C32" s="32" t="str">
         <f aca="false">IF(B26&lt;B25,"OK — mellomleddet reduserer antall kundeforhold","AVVIK: med så få aktører lønner ikke mellomleddet seg på relasjoner alene")</f>
         <v>OK — mellomleddet reduserer antall kundeforhold</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2338,217 +2342,217 @@
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="25" t="n">
         <v>7990000</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="30" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="32" t="n">
-        <f aca="false">B5*B6/365</f>
-        <v>656712.328767123</v>
-      </c>
-      <c r="D7" s="20" t="s">
+      <c r="B7" s="33" t="n">
+        <f aca="false">B5*B6/360</f>
+        <v>665833.333333333</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="26" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="32" t="n">
+      <c r="B9" s="33" t="n">
         <f aca="false">B7*B8</f>
-        <v>65671.2328767123</v>
-      </c>
-      <c r="D9" s="20" t="s">
+        <v>66583.3333333333</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="25" t="n">
         <v>1400000</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="34" t="n">
         <f aca="false">B5/B12</f>
         <v>5.70714285714286</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="21" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="33" t="n">
-        <f aca="false">365/B13</f>
-        <v>63.9549436795995</v>
-      </c>
-      <c r="D14" s="20" t="s">
+      <c r="B14" s="34" t="n">
+        <f aca="false">360/B13</f>
+        <v>63.0788485607009</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="34" t="n">
+      <c r="B15" s="35" t="n">
         <f aca="false">B12*B8</f>
         <v>140000</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="B18" s="29" t="n">
+      <c r="B18" s="30" t="n">
         <v>210</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="26" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="B20" s="24" t="n">
+      <c r="B20" s="25" t="n">
         <v>7300</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B21" s="33" t="n">
+      <c r="B21" s="34" t="n">
         <f aca="false">B18*B19</f>
         <v>42</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="B22" s="32" t="n">
+      <c r="B22" s="33" t="n">
         <f aca="false">B21*B20</f>
         <v>306600</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="21" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="33" t="n">
         <f aca="false">B9+B22</f>
-        <v>372271.232876712</v>
-      </c>
-      <c r="D25" s="20" t="s">
+        <v>373183.333333333</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="C28" s="31" t="str">
-        <f aca="false">IF(ABS(B13*B14-365)&lt;0.01,"OK — omløpshastighet ganger lagringstid er 365 dager","AVVIK: de to tallene henger ikke sammen")</f>
-        <v>OK — omløpshastighet ganger lagringstid er 365 dager</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+      <c r="C28" s="32" t="str">
+        <f aca="false">IF(ABS(B13*B14-360)&lt;0.01,"OK — omløpshastighet ganger lagringstid er 360 dager","AVVIK: de to tallene henger ikke sammen")</f>
+        <v>OK — omløpshastighet ganger lagringstid er 360 dager</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="C29" s="31" t="str">
+      <c r="C29" s="32" t="str">
         <f aca="false">IF(B7&gt;0,"OK — grossisten finansierer en del av driften","AVVIK: uten kredittdager finansierer grossisten ingenting")</f>
         <v>OK — grossisten finansierer en del av driften</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="23" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2581,253 +2585,253 @@
   <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="35" t="n">
         <f aca="false">'Grossistens jobb'!B5</f>
         <v>7990000</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="26" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="32" t="n">
+      <c r="B7" s="33" t="n">
         <f aca="false">B5*B6</f>
         <v>799000</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="B10" s="34" t="n">
+      <c r="B10" s="35" t="n">
         <f aca="false">'Grossistens jobb'!B12</f>
         <v>1400000</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="25" t="n">
         <v>3500000</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="21" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="B12" s="34" t="n">
+      <c r="B12" s="35" t="n">
         <f aca="false">B11-B10</f>
         <v>2100000</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="35" t="n">
         <f aca="false">'Grossistens jobb'!B7</f>
-        <v>656712.328767123</v>
-      </c>
-      <c r="D13" s="20" t="s">
+        <v>665833.333333333</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
         <v>184</v>
       </c>
-      <c r="B14" s="32" t="n">
+      <c r="B14" s="33" t="n">
         <f aca="false">B12+B13</f>
-        <v>2756712.32876712</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+        <v>2765833.33333333</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="28" t="n">
         <f aca="false">'Grossistens jobb'!B8</f>
         <v>0.1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="32" t="n">
+      <c r="B16" s="33" t="n">
         <f aca="false">B14*B15</f>
-        <v>275671.232876712</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
+        <v>276583.333333333</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="25" t="n">
         <v>320000</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="26" t="n">
         <v>0.468</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="B19" s="32" t="n">
+      <c r="B19" s="33" t="n">
         <f aca="false">B17*(1+B18)</f>
         <v>469760</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="21" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="B20" s="32" t="n">
+      <c r="B20" s="33" t="n">
         <f aca="false">'Grossistens jobb'!B22</f>
         <v>306600</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
         <v>192</v>
       </c>
-      <c r="B21" s="32" t="n">
+      <c r="B21" s="33" t="n">
         <f aca="false">B16+B19+B20</f>
-        <v>1052031.23287671</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+        <v>1052943.33333333</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
         <v>194</v>
       </c>
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="33" t="n">
         <f aca="false">B7-B21</f>
-        <v>-253031.232876712</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+        <v>-253943.333333334</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="35" t="n">
+      <c r="B25" s="36" t="n">
         <f aca="false">B21/B5</f>
-        <v>0.131668489721741</v>
-      </c>
-      <c r="D25" s="20" t="s">
+        <v>0.131782644972883</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="D26" s="36" t="str">
+      <c r="D26" s="37" t="str">
         <f aca="false">IF(B24&gt;0,"Direkte innkjøp lønner seg med disse forutsetningene","Rabatten er ekte, men den er ikke stor nok. Grossisten gjør en jobb Nordlys måtte gjort selv")</f>
         <v>Rabatten er ekte, men den er ikke stor nok. Grossisten gjør en jobb Nordlys måtte gjort selv</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="31" t="str">
+      <c r="C29" s="32" t="str">
         <f aca="false">IF(ABS(B21-(B16+B19+B20))&lt;0.01,"OK — de tre kostnadslinjene summerer seg til sum ekstrakostnader","AVVIK: summen stemmer ikke med linjene over")</f>
         <v>OK — de tre kostnadslinjene summerer seg til sum ekstrakostnader</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="C30" s="31" t="str">
+      <c r="C30" s="32" t="str">
         <f aca="false">IF(B6&gt;=B25,"OK — rabatten dekker ekstrakostnadene","AVVIK: rabatten er lavere enn den rabatten som gir balanse. Direkte innkjøp taper penger med dagens volum")</f>
         <v>AVVIK: rabatten er lavere enn den rabatten som gir balanse. Direkte innkjøp taper penger med dagens volum</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="C32" s="31" t="str">
+      <c r="C32" s="32" t="str">
         <f aca="false">IF(ABS(B14-(B12+B13))&lt;0.01,"OK — kapitalbindingen er økt lager pluss bortfalt kreditt","AVVIK: kapitalbindingen stemmer ikke")</f>
         <v>OK — kapitalbindingen er økt lager pluss bortfalt kreditt</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
         <v>202</v>
       </c>
     </row>
@@ -2865,553 +2869,553 @@
   <dimension ref="A1:E68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="54"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="28" t="n">
         <f aca="false">'Direkte innkjøp'!B10/'Direkte innkjøp'!B5</f>
         <v>0.175219023779725</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="28" t="n">
         <f aca="false">'Direkte innkjøp'!B11/'Direkte innkjøp'!B5</f>
         <v>0.438047559449312</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="B9" s="27" t="n">
-        <f aca="false">'Grossistens jobb'!B6/365</f>
-        <v>0.0821917808219178</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
+      <c r="B9" s="28" t="n">
+        <f aca="false">'Grossistens jobb'!B6/360</f>
+        <v>0.0833333333333333</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
         <v>210</v>
       </c>
-      <c r="B10" s="37" t="n">
+      <c r="B10" s="38" t="n">
         <f aca="false">B8-B7+B9</f>
-        <v>0.345020316491505</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
+        <v>0.34616186900292</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
         <v>211</v>
       </c>
-      <c r="B11" s="35" t="n">
+      <c r="B11" s="36" t="n">
         <f aca="false">'Direkte innkjøp'!B6-B10*'Direkte innkjøp'!B15</f>
-        <v>0.0654979683508495</v>
-      </c>
-      <c r="E11" s="20" t="s">
+        <v>0.065383813099708</v>
+      </c>
+      <c r="E11" s="21" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
         <v>213</v>
       </c>
-      <c r="B12" s="32" t="n">
+      <c r="B12" s="33" t="n">
         <f aca="false">'Direkte innkjøp'!B19+'Direkte innkjøp'!B20</f>
         <v>776360</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="21" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
         <v>215</v>
       </c>
-      <c r="B13" s="32" t="n">
+      <c r="B13" s="33" t="n">
         <f aca="false">IF(B11&lt;=0,"finnes ikke",B12/B11)</f>
-        <v>11853192.0843913</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+        <v>11873886.8719094</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="B14" s="34" t="n">
+      <c r="B14" s="35" t="n">
         <f aca="false">'Direkte innkjøp'!B5</f>
         <v>7990000</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
         <v>217</v>
       </c>
-      <c r="B15" s="37" t="n">
+      <c r="B15" s="38" t="n">
         <f aca="false">IF(B11&lt;=0,"",B13/B14-1)</f>
-        <v>0.483503389786142</v>
+        <v>0.486093475833466</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="24" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="35" t="n">
         <f aca="false">B18*$B$14</f>
         <v>3995000</v>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="26" t="n">
         <v>0.5</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="35" t="n">
         <f aca="false">A18*$B$11</f>
-        <v>261664.383561644</v>
-      </c>
-      <c r="D18" s="34" t="n">
+        <v>261208.333333333</v>
+      </c>
+      <c r="D18" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E18" s="32" t="n">
+      <c r="E18" s="33" t="n">
         <f aca="false">C18-D18</f>
-        <v>-514695.616438356</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34" t="n">
+        <v>-515151.666666667</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="35" t="n">
         <f aca="false">B19*$B$14</f>
         <v>5992500</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="26" t="n">
         <v>0.75</v>
       </c>
-      <c r="C19" s="34" t="n">
+      <c r="C19" s="35" t="n">
         <f aca="false">A19*$B$11</f>
-        <v>392496.575342466</v>
-      </c>
-      <c r="D19" s="34" t="n">
+        <v>391812.5</v>
+      </c>
+      <c r="D19" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E19" s="32" t="n">
+      <c r="E19" s="33" t="n">
         <f aca="false">C19-D19</f>
-        <v>-383863.424657534</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="n">
+        <v>-384547.5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="35" t="n">
         <f aca="false">B20*$B$14</f>
         <v>7990000</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="34" t="n">
+      <c r="C20" s="35" t="n">
         <f aca="false">A20*$B$11</f>
-        <v>523328.767123288</v>
-      </c>
-      <c r="D20" s="34" t="n">
+        <v>522416.666666667</v>
+      </c>
+      <c r="D20" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E20" s="32" t="n">
+      <c r="E20" s="33" t="n">
         <f aca="false">C20-D20</f>
-        <v>-253031.232876712</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="n">
+        <v>-253943.333333333</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="35" t="n">
         <f aca="false">B21*$B$14</f>
         <v>9987500</v>
       </c>
-      <c r="B21" s="25" t="n">
+      <c r="B21" s="26" t="n">
         <v>1.25</v>
       </c>
-      <c r="C21" s="34" t="n">
+      <c r="C21" s="35" t="n">
         <f aca="false">A21*$B$11</f>
-        <v>654160.95890411</v>
-      </c>
-      <c r="D21" s="34" t="n">
+        <v>653020.833333333</v>
+      </c>
+      <c r="D21" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E21" s="32" t="n">
+      <c r="E21" s="33" t="n">
         <f aca="false">C21-D21</f>
-        <v>-122199.04109589</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="n">
+        <v>-123339.166666667</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="35" t="n">
         <f aca="false">B22*$B$14</f>
         <v>11985000</v>
       </c>
-      <c r="B22" s="25" t="n">
+      <c r="B22" s="26" t="n">
         <v>1.5</v>
       </c>
-      <c r="C22" s="34" t="n">
+      <c r="C22" s="35" t="n">
         <f aca="false">A22*$B$11</f>
-        <v>784993.150684932</v>
-      </c>
-      <c r="D22" s="34" t="n">
+        <v>783625</v>
+      </c>
+      <c r="D22" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E22" s="32" t="n">
+      <c r="E22" s="33" t="n">
         <f aca="false">C22-D22</f>
-        <v>8633.15068493167</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="n">
+        <v>7265.00000000012</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="35" t="n">
         <f aca="false">B23*$B$14</f>
         <v>13982500</v>
       </c>
-      <c r="B23" s="25" t="n">
+      <c r="B23" s="26" t="n">
         <v>1.75</v>
       </c>
-      <c r="C23" s="34" t="n">
+      <c r="C23" s="35" t="n">
         <f aca="false">A23*$B$11</f>
-        <v>915825.342465754</v>
-      </c>
-      <c r="D23" s="34" t="n">
+        <v>914229.166666667</v>
+      </c>
+      <c r="D23" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E23" s="32" t="n">
+      <c r="E23" s="33" t="n">
         <f aca="false">C23-D23</f>
-        <v>139465.342465754</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="n">
+        <v>137869.166666667</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="35" t="n">
         <f aca="false">B24*$B$14</f>
         <v>15980000</v>
       </c>
-      <c r="B24" s="25" t="n">
+      <c r="B24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="34" t="n">
+      <c r="C24" s="35" t="n">
         <f aca="false">A24*$B$11</f>
-        <v>1046657.53424658</v>
-      </c>
-      <c r="D24" s="34" t="n">
+        <v>1044833.33333333</v>
+      </c>
+      <c r="D24" s="35" t="n">
         <f aca="false">$B$12</f>
         <v>776360</v>
       </c>
-      <c r="E24" s="32" t="n">
+      <c r="E24" s="33" t="n">
         <f aca="false">C24-D24</f>
-        <v>270297.534246576</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+        <v>268473.333333334</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="C27" s="31" t="str">
+      <c r="C27" s="32" t="str">
         <f aca="false">IF(ABS($B$14*$B$11-$B$12-'Direkte innkjøp'!B24)&lt;1,"OK — vendepunktsmodellen gir samme netto som oppstillingen","AVVIK: modellen og oppstillingen er ikke enige")</f>
         <v>OK — vendepunktsmodellen gir samme netto som oppstillingen</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="C28" s="31" t="str">
+      <c r="C28" s="32" t="str">
         <f aca="false">IF(NOT(ISNUMBER($B$13)),"AVVIK: rabatten dekker ikke engang kapitalkostnaden. Da finnes det ikke noe vendepunkt",IF($B$13&gt;$B$14,"OK — direkte innkjøp lønner seg først ved et større materiellvolum enn Nordlys har i dag","AVVIK: da lønner direkte innkjøp seg allerede"))</f>
         <v>OK — direkte innkjøp lønner seg først ved et større materiellvolum enn Nordlys har i dag</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="C29" s="31" t="str">
+      <c r="C29" s="32" t="str">
         <f aca="false">IF(AND(E18&lt;0,E24&gt;0),"OK — tabellen snur fra tap til gevinst, og vendepunktet ligger et sted imellom","AVVIK: utvid volumtrappen så vendepunktet kommer med")</f>
         <v>OK — tabellen snur fra tap til gevinst, og vendepunktet ligger et sted imellom</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="B35" s="25" t="n">
+      <c r="B35" s="26" t="n">
         <v>0.03</v>
       </c>
-      <c r="E35" s="20" t="s">
+      <c r="E35" s="21" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="B36" s="24" t="n">
+      <c r="B36" s="25" t="n">
         <v>2600000</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="B37" s="34" t="n">
+      <c r="B37" s="35" t="n">
         <f aca="false">'Direkte innkjøp'!B10</f>
         <v>1400000</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="23" t="s">
         <v>181</v>
       </c>
-      <c r="B38" s="32" t="n">
+      <c r="B38" s="33" t="n">
         <f aca="false">B36-B37</f>
         <v>1200000</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="19" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="22" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="B41" s="32" t="n">
+      <c r="B41" s="33" t="n">
         <f aca="false">'Direkte innkjøp'!B5*B35</f>
         <v>239700</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="19" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="20" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="B44" s="34" t="n">
+      <c r="B44" s="35" t="n">
         <f aca="false">B38*'Direkte innkjøp'!B15</f>
         <v>120000</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="B45" s="25" t="n">
+      <c r="B45" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="E45" s="20" t="s">
+      <c r="E45" s="21" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="B46" s="34" t="n">
+      <c r="B46" s="35" t="n">
         <f aca="false">B38*B45</f>
         <v>72000</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="22" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="B47" s="32" t="n">
+      <c r="B47" s="33" t="n">
         <f aca="false">B44+B46</f>
         <v>192000</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="19" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="22" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="23" t="s">
         <v>240</v>
       </c>
-      <c r="B50" s="32" t="n">
+      <c r="B50" s="33" t="n">
         <f aca="false">B41-B47</f>
         <v>47700</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="20" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B51" s="38" t="n">
+      <c r="B51" s="39" t="n">
         <f aca="false">B47/'Direkte innkjøp'!B5</f>
         <v>0.0240300375469337</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="20" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="B52" s="27" t="n">
+      <c r="B52" s="28" t="n">
         <f aca="false">1-B47/(B41)</f>
         <v>0.198998748435544</v>
       </c>
-      <c r="E52" s="20" t="s">
+      <c r="E52" s="21" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="20" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="B53" s="39" t="n">
-        <f aca="false">365/('Direkte innkjøp'!B5/B36)</f>
-        <v>118.773466833542</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="20" t="s">
+      <c r="B53" s="40" t="n">
+        <f aca="false">360/('Direkte innkjøp'!B5/B36)</f>
+        <v>117.146433041302</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="B54" s="39" t="n">
+      <c r="B54" s="40" t="n">
         <f aca="false">'Grossistens jobb'!B14</f>
-        <v>63.9549436795995</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="18" t="s">
+        <v>63.0788485607009</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="19" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="20" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="B57" s="25" t="n">
+      <c r="B57" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="E57" s="20" t="s">
+      <c r="E57" s="21" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="20" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="B58" s="34" t="n">
+      <c r="B58" s="35" t="n">
         <f aca="false">B38*B57</f>
         <v>60000</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="22" t="s">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="B59" s="32" t="n">
+      <c r="B59" s="33" t="n">
         <f aca="false">B50-B58</f>
         <v>-12300</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="20" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="E60" s="36" t="str">
+      <c r="E60" s="37" t="str">
         <f aca="false">IF(B50&lt;=0,"Avtalen bærer ikke engang på papiret. Si nei",IF(B59&lt;=0,"Avtalen bærer på papiret, men ikke når risikoen for ukurans tas med. Forhandle om høyere rabatt eller returrett","Avtalen bærer også med ukurans. Si ja, men mål lagringstiden"))</f>
         <v>Avtalen bærer på papiret, men ikke når risikoen for ukurans tas med. Forhandle om høyere rabatt eller returrett</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="18" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="19" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="20" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="21" t="s">
         <v>250</v>
       </c>
-      <c r="C63" s="31" t="str">
+      <c r="C63" s="32" t="str">
         <f aca="false">IF(B50&gt;0,"OK — rabatten er større enn kostnaden ved å holde lageret selv","AVVIK: rabatten dekker ikke engang kapital og lagerhold")</f>
         <v>OK — rabatten er større enn kostnaden ved å holde lageret selv</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="20" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="C64" s="31" t="str">
+      <c r="C64" s="32" t="str">
         <f aca="false">IF(B59&gt;0,"OK — avtalen bærer også med ukurans","AVVIK: avtalen snur til tap så snart noe av det ekstra lageret blir liggende. Det er selve poenget i oppgaven")</f>
         <v>AVVIK: avtalen snur til tap så snart noe av det ekstra lageret blir liggende. Det er selve poenget i oppgaven</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="17" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="20" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="21" t="s">
         <v>253</v>
       </c>
-      <c r="C66" s="31" t="str">
+      <c r="C66" s="32" t="str">
         <f aca="false">IF(B53&gt;B54,"OK — et større lager gir lengre lagringstid, og lengre lagringstid gir større risiko for ukurans","AVVIK: kontroller lagertallene")</f>
         <v>OK — et større lager gir lengre lagringstid, og lengre lagringstid gir større risiko for ukurans</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="17" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="18" t="s">
         <v>254</v>
       </c>
     </row>

</xml_diff>